<commit_message>
criação e finalização do projeto ReadExcelGifText
</commit_message>
<xml_diff>
--- a/ReadExcelGifText/src/Images/Output.xlsx
+++ b/ReadExcelGifText/src/Images/Output.xlsx
@@ -11,15 +11,51 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
-    <t>Url Do Gif</t>
+    <t>Path on computer</t>
   </si>
   <si>
-    <t>Caminho do URL (Opctional)</t>
+    <t>Path of URL (Opctional)</t>
   </si>
   <si>
-    <t>Tempo de Loading</t>
+    <t>Time of Loading</t>
+  </si>
+  <si>
+    <t>https://media1.tenor.com/m/ilxUzeIvTtcAAAAd/moo-moo-mario-kart.gif</t>
+  </si>
+  <si>
+    <t>4.722</t>
+  </si>
+  <si>
+    <t>https://media1.tenor.com/m/8pgQSVm9PQ4AAAAd/mario-kart-world-mario-kart.gif</t>
+  </si>
+  <si>
+    <t>2.42</t>
+  </si>
+  <si>
+    <t>https://media1.tenor.com/m/04KL5cq4sakAAAAd/mario-kart-world-nintendo-switch-2.gif</t>
+  </si>
+  <si>
+    <t>1.121</t>
+  </si>
+  <si>
+    <t>https://media1.tenor.com/m/cKQMcytrcpAAAAAd/ptooie-blowing.gif</t>
+  </si>
+  <si>
+    <t>1.064</t>
+  </si>
+  <si>
+    <t>https://media1.tenor.com/m/pClBfwj7yVcAAAAd/touring-peach-princess-peach.gif</t>
+  </si>
+  <si>
+    <t>1.907</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>undefined</t>
   </si>
 </sst>
 </file>
@@ -65,7 +101,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
     <row r="2" spans="3:5">
@@ -79,6 +115,54 @@
         <v>2</v>
       </c>
     </row>
+    <row r="3" spans="4:5">
+      <c r="D3" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="4:5">
+      <c r="D4" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="4:5">
+      <c r="D5" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="4:5">
+      <c r="D6" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="4:5">
+      <c r="D7" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="3:5">
+      <c r="C8" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>